<commit_message>
update flow provider map, integrate swolfpy and warm flow libraries
</commit_message>
<xml_diff>
--- a/wmlci/utils/flowmapping/SwolfPy_WTE_Tech_flow_map.xlsx
+++ b/wmlci/utils/flowmapping/SwolfPy_WTE_Tech_flow_map.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hwatson\code\environments\general\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hwatson\code\environments\WMLCI\wmlci\utils\flowmapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C673572-8665-4A1D-B377-02544B498CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F72AD3-C851-4F97-8478-B395BD25E4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{97F67A38-5F43-40D8-AB89-1621D7974266}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>ammonia_liquid_RoW_ammonia_production_steam_reforming_liquid</t>
   </si>
@@ -57,18 +56,6 @@
     <t>lime_hydrated_loose_weight_RoW_lime_production</t>
   </si>
   <si>
-    <t>Transport, combination truck; diesel powered</t>
-  </si>
-  <si>
-    <t>34156f3c-28ef-33db-9ad0-6293a2aa0d52</t>
-  </si>
-  <si>
-    <t>Charcoal; at plant</t>
-  </si>
-  <si>
-    <t>1f6ba8b1-eff7-4dd9-b73c-b29330a15daf</t>
-  </si>
-  <si>
     <t>Cutoff flow</t>
   </si>
   <si>
@@ -93,18 +80,6 @@
     <t>USLCI Flow Provider UUID</t>
   </si>
   <si>
-    <t>628c07ec-0802-39c1-ab88-1c62848ef436</t>
-  </si>
-  <si>
-    <t>Transport; combination truck; diesel powered</t>
-  </si>
-  <si>
-    <t>Hydrated lime; at plant</t>
-  </si>
-  <si>
-    <t>11d7c675-cf33-4cde-b5c7-e42ce2ed8c61</t>
-  </si>
-  <si>
     <t>072a4586-44d6-3428-a15c-8e1e8a0031cc</t>
   </si>
   <si>
@@ -154,6 +129,45 @@
   </si>
   <si>
     <t>03f7870f-062a-3dd1-b3ec-1566c69918b8</t>
+  </si>
+  <si>
+    <t>Transport; single unit truck, short-haul; diesel powered</t>
+  </si>
+  <si>
+    <t>20567d69-c8ee-325c-a98c-43c35b8eb9f4</t>
+  </si>
+  <si>
+    <t>Transport, single unit truck; short-haul; diesel powered</t>
+  </si>
+  <si>
+    <t>711ab26a-94a2-33f9-89da-560c55808297</t>
+  </si>
+  <si>
+    <t>Electricity; at user; consumption mix - US - US</t>
+  </si>
+  <si>
+    <t>75d4be66-12a7-30b3-bc57-fa724c941b0e</t>
+  </si>
+  <si>
+    <t>Quicklime; at plant</t>
+  </si>
+  <si>
+    <t>9c0c2415-126f-3162-8479-f002f315a8c7</t>
+  </si>
+  <si>
+    <t>c34c4451-297f-3b5c-a15f-2c16cdb52ad9</t>
+  </si>
+  <si>
+    <t>Granular activated carbon production; at plant - PROXY</t>
+  </si>
+  <si>
+    <t>b0d4a167-e4f4-3ecd-8ce0-76caf610a6ff</t>
+  </si>
+  <si>
+    <t>Granular activated carbon; at plant</t>
+  </si>
+  <si>
+    <t>6e14dcda-bea9-327c-b43d-e4cacbecca2f</t>
   </si>
 </sst>
 </file>
@@ -544,7 +558,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -562,174 +576,174 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="K1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="L1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
         <v>28</v>
       </c>
-      <c r="H2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" t="s">
-        <v>36</v>
-      </c>
       <c r="L2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" t="s">
-        <v>37</v>
-      </c>
       <c r="L3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I4" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="J4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I5" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="J5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L5" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>